<commit_message>
docs: complete E2E test evidence with 28 screenshots and execution logs
</commit_message>
<xml_diff>
--- a/docs/GoogleDrive_Upload/成果物一覧/Mauro_Brenda_Taxi_Link_成果物一覧.xlsx
+++ b/docs/GoogleDrive_Upload/成果物一覧/Mauro_Brenda_Taxi_Link_成果物一覧.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="プロジェクト概要" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成果物サマリー" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="成果物一覧" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -515,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C11"/>
+  <dimension ref="B2:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -532,7 +532,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>プロジェクト成果物一覧（Deliverables Inventory）</t>
+          <t>プロジェクト納品成果物一覧 ＆ 構成インベントリ</t>
         </is>
       </c>
     </row>
@@ -544,14 +544,14 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Mauro &amp; Brenda Taxi Link (英語教室 送迎チケット管理)</t>
+          <t>Mauro &amp; Brenda Taxi Link (英語教室 送迎チケット管理Webアプリケーション)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>公開WebサイトURL</t>
+          <t>公開WebアプリURL</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -563,7 +563,7 @@
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>ソースコードリポジトリ</t>
+          <t>GitHubリポジトリ</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -575,7 +575,7 @@
     <row r="8">
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>主要関係者</t>
+          <t>主な関係者</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -587,36 +587,48 @@
     <row r="9">
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>納品日 / バージョン</t>
+          <t>納品日</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>2026年10月08日 / v1.0.0 (プロダクションリリース)</t>
+          <t>2026年10月08日</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>開発技術スタック</t>
+          <t>成果物合計</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>React 19, TypeScript, Tailwind CSS, Vite, GitHub Pages, Google Apps Script</t>
+          <t>全15点（システム本体 3点 / バックエンド・連携 3点 / 仕様書 3点 / テスト・証跡 4点 / ガイド 2点）</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>主要機能</t>
+          <t>受入テスト結果</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>管理者・保護者の2軸UI、片道1枚消費ルール、フレックス予約、チケット残少連絡アラート、GAS自動連携</t>
+          <t>全28項目 100% PASS（全件の実行ログ・画面キャプチャー証跡完備）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Googleドライブ保管先</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/u/0/folders/1k1HwCo8p37e1Vpm6Qu2ZGPxGfAhbWFzx</t>
         </is>
       </c>
     </row>
@@ -631,16 +643,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G16"/>
+  <dimension ref="A2:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="2" ht="28" customHeight="1">
@@ -680,7 +692,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="26" customHeight="1">
+    <row r="3" ht="28" customHeight="1">
       <c r="A3" s="6" t="n">
         <v>1</v>
       </c>
@@ -715,7 +727,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="26" customHeight="1">
+    <row r="4" ht="28" customHeight="1">
       <c r="A4" s="9" t="n">
         <v>2</v>
       </c>
@@ -750,7 +762,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="26" customHeight="1">
+    <row r="5" ht="28" customHeight="1">
       <c r="A5" s="6" t="n">
         <v>3</v>
       </c>
@@ -785,7 +797,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="26" customHeight="1">
+    <row r="6" ht="28" customHeight="1">
       <c r="A6" s="9" t="n">
         <v>4</v>
       </c>
@@ -820,7 +832,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="26" customHeight="1">
+    <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6" t="n">
         <v>5</v>
       </c>
@@ -841,7 +853,7 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>「生徒台帳」「送迎履歴」「チケット購入履歴」の3テーブルスキーマ定義および自動データ同期インターフェース</t>
+          <t>「生徒台帳」「送迎予定履歴」「チケット購入履歴」の3テーブルスキーマ定義および自動データ同期インターフェース</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -855,7 +867,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="26" customHeight="1">
+    <row r="8" ht="28" customHeight="1">
       <c r="A8" s="9" t="n">
         <v>6</v>
       </c>
@@ -890,7 +902,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="26" customHeight="1">
+    <row r="9" ht="28" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>7</v>
       </c>
@@ -925,7 +937,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="26" customHeight="1">
+    <row r="10" ht="28" customHeight="1">
       <c r="A10" s="9" t="n">
         <v>8</v>
       </c>
@@ -960,7 +972,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="26" customHeight="1">
+    <row r="11" ht="28" customHeight="1">
       <c r="A11" s="6" t="n">
         <v>9</v>
       </c>
@@ -995,7 +1007,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="26" customHeight="1">
+    <row r="12" ht="28" customHeight="1">
       <c r="A12" s="9" t="n">
         <v>10</v>
       </c>
@@ -1016,7 +1028,7 @@
       </c>
       <c r="E12" s="10" t="inlineStr">
         <is>
-          <t>保護者ポータル・先生ダッシュボード・Google連携・レスポンシブの全28項目テストマトリクス（合否チェックリスト付）</t>
+          <t>保護者ポータル・先生ダッシュボード・Google連携・レスポンシブの全28項目テストマトリクス（合否・証跡ファイル名・実行ログ付）</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
@@ -1026,11 +1038,11 @@
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>完了（Pass）</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="26" customHeight="1">
+          <t>完了（Pass 100%）</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
       <c r="A13" s="6" t="n">
         <v>11</v>
       </c>
@@ -1051,7 +1063,7 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>全28項目の操作手順、前提条件、期待される結果、判定結果を美麗にスタイリングした配布・印刷用PDF</t>
+          <t>全28項目の操作手順、前提条件、期待される結果、証跡ファイル、E2Eログを収録した配布・印刷用PDF</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -1061,11 +1073,11 @@
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>完了（Pass）</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="26" customHeight="1">
+          <t>完了（Pass 100%）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
       <c r="A14" s="9" t="n">
         <v>12</v>
       </c>
@@ -1076,66 +1088,66 @@
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>自動スクリーンショット &amp; E2E検証スクリプト</t>
+          <t>受入テスト客観的証跡一式 (キャプチャー＆ログ)</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>Node.js (Puppeteer)</t>
+          <t>PNG 28枚 + TXTログ</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
         <is>
-          <t>PC・スマホ両解像度での全画面自動キャプチャーおよびデータ同期検証を行う自動化スクリプト</t>
+          <t>全28テストケースの自動ブラウザ実行時のスクリーンショット（docs/evidence/TC-xxx.png）および詳細実行ログ（test_execution_log.txt）</t>
         </is>
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>開発者</t>
+          <t>全関係者・受入確認者</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>完了（検証済）</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="26" customHeight="1">
+          <t>完了（全28件完備）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
       <c r="A15" s="6" t="n">
         <v>13</v>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>運用マニュアル</t>
+          <t>テスト・品質検証</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Google連携導入4ステップガイド</t>
+          <t>全自動E2E証跡取得テストスイート</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Web内蔵ガイド</t>
+          <t>Node.js (Puppeteer)</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Googleスプレッドシート新規作成からGASデプロイ、WebアプリURL貼り付けまでの手順をWeb画面内にわかりやすく内蔵</t>
+          <t>全28ケースを自動実行し、DOM値・ダイアログ処理・画面キャプチャー・ログをリアルタイム採取するテストエンジン (scripts/run_all_e2e_evidence.cjs)</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Mauro・Brenda先生、小林様</t>
+          <t>開発者・品質保証</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>完了（Web画面内）</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="26" customHeight="1">
+          <t>完了（動作検証済）</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
       <c r="A16" s="9" t="n">
         <v>14</v>
       </c>
@@ -1146,25 +1158,60 @@
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>成果物一覧ファイル一式</t>
+          <t>Google連携導入4ステップガイド</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Excel / PDF / Markdown</t>
+          <t>Web内蔵ガイド</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>納品・共有対象となるすべての成果物とその所在・ステータスをまとめたインベントリ（本ファイル群）</t>
+          <t>Googleスプレッドシート新規作成からGASデプロイ、WebアプリURL貼り付けまでの手順をWeb画面内にわかりやすく内蔵</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>全関係者</t>
+          <t>Mauro・Brenda先生、小林様</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>完了（Web画面内）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>運用マニュアル</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>システム管理者・利用者運用手引書</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Markdown / ドキュメント</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>日常の送迎受付、チケット追加チャージ、急な予定変更・キャンセル、トラブルシューティングの手順</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Mauro・Brenda先生、保護者</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
         <is>
           <t>完了</t>
         </is>

</xml_diff>